<commit_message>
Refactor/add xlsx interface sheet
</commit_message>
<xml_diff>
--- a/cea_model.xlsx
+++ b/cea_model.xlsx
@@ -16,6 +16,7 @@
     <sheet name="Transition matrix" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Results" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="Charts" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Interface" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="cohort_size">'Inputs'!$B$6</definedName>
@@ -2629,7 +2630,7 @@
     <from>
       <col>1</col>
       <colOff>0</colOff>
-      <row>30</row>
+      <row>31</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="6240780" cy="3053524"/>
@@ -3058,7 +3059,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:C75"/>
+  <dimension ref="B1:C76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -3313,288 +3314,300 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="22" customHeight="1">
-      <c r="B30" s="3" t="inlineStr">
+    <row r="29" ht="16.5" customHeight="1">
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Interface</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>For programs that run the workbook: which cells are its inputs and results. You do not need it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="22" customHeight="1">
+      <c r="B31" s="3" t="inlineStr">
         <is>
           <t>The model</t>
         </is>
       </c>
     </row>
-    <row r="49" ht="22" customHeight="1">
-      <c r="B49" s="3" t="inlineStr">
+    <row r="50" ht="22" customHeight="1">
+      <c r="B50" s="3" t="inlineStr">
         <is>
           <t>Key ideas</t>
         </is>
       </c>
     </row>
-    <row r="50" ht="30" customHeight="1">
-      <c r="B50" s="5" t="inlineStr">
+    <row r="51" ht="30" customHeight="1">
+      <c r="B51" s="5" t="inlineStr">
         <is>
           <t>Markov cohort model</t>
         </is>
       </c>
-      <c r="C50" s="4" t="inlineStr">
+      <c r="C51" s="4" t="inlineStr">
         <is>
           <t>Instead of simulating people one by one, it tracks how many people of a group are in each health state, and moves them between states once per cycle.</t>
         </is>
       </c>
     </row>
-    <row r="51" ht="16.5" customHeight="1">
-      <c r="B51" s="5" t="inlineStr">
+    <row r="52" ht="16.5" customHeight="1">
+      <c r="B52" s="5" t="inlineStr">
         <is>
           <t>Cycle</t>
         </is>
       </c>
-      <c r="C51" s="4" t="inlineStr">
+      <c r="C52" s="4" t="inlineStr">
         <is>
           <t>The time step of the model: here one year, so one row of a Trace sheet.</t>
         </is>
       </c>
     </row>
-    <row r="52" ht="30" customHeight="1">
-      <c r="B52" s="5" t="inlineStr">
+    <row r="53" ht="30" customHeight="1">
+      <c r="B53" s="5" t="inlineStr">
         <is>
           <t>Transition probability</t>
         </is>
       </c>
-      <c r="C52" s="4" t="inlineStr">
+      <c r="C53" s="4" t="inlineStr">
         <is>
           <t>The chance of moving from one state to another in one cycle, for example from Healthy to Early cancer.</t>
         </is>
       </c>
     </row>
-    <row r="53" ht="43.5" customHeight="1">
-      <c r="B53" s="5" t="inlineStr">
+    <row r="54" ht="43.5" customHeight="1">
+      <c r="B54" s="5" t="inlineStr">
         <is>
           <t>Transition matrix</t>
         </is>
       </c>
-      <c r="C53" s="4" t="inlineStr">
+      <c r="C54" s="4" t="inlineStr">
         <is>
           <t>All the transition probabilities in a table: one row per state now, one column per state a year later. Each row adds up to 1. Here it changes with age and with screening, so each row of a Trace sheet has its own.</t>
         </is>
       </c>
     </row>
-    <row r="54" ht="16.5" customHeight="1">
-      <c r="B54" s="5" t="inlineStr">
+    <row r="55" ht="16.5" customHeight="1">
+      <c r="B55" s="5" t="inlineStr">
         <is>
           <t>Markov trace</t>
         </is>
       </c>
-      <c r="C54" s="4" t="inlineStr">
+      <c r="C55" s="4" t="inlineStr">
         <is>
           <t>The number of people in each state, cycle after cycle.</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="30" customHeight="1">
-      <c r="B55" s="5" t="inlineStr">
-        <is>
-          <t>Utility and QALY</t>
-        </is>
-      </c>
-      <c r="C55" s="4" t="inlineStr">
-        <is>
-          <t>A utility weights a year by its quality of life (1 = full health, 0 = dead). A quality-adjusted life year (QALY) is a year lived times its utility.</t>
         </is>
       </c>
     </row>
     <row r="56" ht="30" customHeight="1">
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>Discounting</t>
+          <t>Utility and QALY</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>Costs and health in the future are valued less than now. A value in year t is multiplied by 1 / (1 + rate)^t.</t>
+          <t>A utility weights a year by its quality of life (1 = full health, 0 = dead). A quality-adjusted life year (QALY) is a year lived times its utility.</t>
         </is>
       </c>
     </row>
     <row r="57" ht="30" customHeight="1">
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>ICER</t>
+          <t>Discounting</t>
         </is>
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>Incremental cost-effectiveness ratio: the extra cost of a strategy divided by the extra QALYs it gives, compared with an alternative. "€ per QALY gained".</t>
+          <t>Costs and health in the future are valued less than now. A value in year t is multiplied by 1 / (1 + rate)^t.</t>
         </is>
       </c>
     </row>
     <row r="58" ht="30" customHeight="1">
       <c r="B58" s="5" t="inlineStr">
         <is>
-          <t>Willingness to pay</t>
+          <t>ICER</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>The threshold: the most a health system pays per QALY gained. A strategy with an ICER below it is considered cost-effective.</t>
+          <t>Incremental cost-effectiveness ratio: the extra cost of a strategy divided by the extra QALYs it gives, compared with an alternative. "€ per QALY gained".</t>
         </is>
       </c>
     </row>
     <row r="59" ht="30" customHeight="1">
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>Dominance</t>
+          <t>Willingness to pay</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>A strategy is dominated if another one is cheaper and gives more QALYs. It is extendedly dominated if a mix of two others would beat it.</t>
+          <t>The threshold: the most a health system pays per QALY gained. A strategy with an ICER below it is considered cost-effective.</t>
         </is>
       </c>
     </row>
     <row r="60" ht="30" customHeight="1">
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>Efficiency frontier</t>
+          <t>Dominance</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>The strategies that are not dominated, sorted by cost. ICERs are calculated along it, each strategy against the previous one.</t>
+          <t>A strategy is dominated if another one is cheaper and gives more QALYs. It is extendedly dominated if a mix of two others would beat it.</t>
         </is>
       </c>
     </row>
     <row r="61" ht="30" customHeight="1">
       <c r="B61" s="5" t="inlineStr">
         <is>
+          <t>Efficiency frontier</t>
+        </is>
+      </c>
+      <c r="C61" s="4" t="inlineStr">
+        <is>
+          <t>The strategies that are not dominated, sorted by cost. ICERs are calculated along it, each strategy against the previous one.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="30" customHeight="1">
+      <c r="B62" s="5" t="inlineStr">
+        <is>
           <t>Net monetary benefit</t>
         </is>
       </c>
-      <c r="C61" s="4" t="inlineStr">
+      <c r="C62" s="4" t="inlineStr">
         <is>
           <t>QALYs x willingness to pay - cost. The strategy with the highest one is the cost-effective choice; it always agrees with the frontier.</t>
         </is>
       </c>
     </row>
-    <row r="63" ht="22" customHeight="1">
-      <c r="B63" s="3" t="inlineStr">
+    <row r="64" ht="22" customHeight="1">
+      <c r="B64" s="3" t="inlineStr">
         <is>
           <t>Things to try</t>
-        </is>
-      </c>
-    </row>
-    <row r="64" ht="30" customHeight="1">
-      <c r="B64" s="5" t="inlineStr">
-        <is>
-          <t>Exercise 1</t>
-        </is>
-      </c>
-      <c r="C64" s="4" t="inlineStr">
-        <is>
-          <t>Set screening participation to 100%. How many more cancer deaths are avoided (Results, section 5)? Does the ICER of screening get better or worse?</t>
         </is>
       </c>
     </row>
     <row r="65" ht="30" customHeight="1">
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>Exercise 2</t>
+          <t>Exercise 1</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>Strategy 3 (from 45) is just above the willingness to pay. Raise the willingness to pay until it becomes the cost-effective strategy. Compare your answer with its ICER in Results, section 3.</t>
+          <t>Set screening participation to 100%. How many more cancer deaths are avoided (Results, section 5)? Does the ICER of screening get better or worse?</t>
         </is>
       </c>
     </row>
     <row r="66" ht="30" customHeight="1">
       <c r="B66" s="5" t="inlineStr">
         <is>
-          <t>Exercise 3</t>
+          <t>Exercise 2</t>
         </is>
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>Set both discount rates to 0%. Why does screening look better? (Hint: when are its costs paid, and when are its benefits enjoyed?)</t>
+          <t>Strategy 3 (from 45) is just above the willingness to pay. Raise the willingness to pay until it becomes the cost-effective strategy. Compare your answer with its ICER in Results, section 3.</t>
         </is>
       </c>
     </row>
     <row r="67" ht="30" customHeight="1">
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>Exercise 4</t>
+          <t>Exercise 3</t>
         </is>
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>Make the test perfect (sensitivity and specificity 100%). What happens to the cost of screening (Results, section 4), and to the status of "No screening" in section 3? Why?</t>
+          <t>Set both discount rates to 0%. Why does screening look better? (Hint: when are its costs paid, and when are its benefits enjoyed?)</t>
         </is>
       </c>
     </row>
     <row r="68" ht="30" customHeight="1">
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>Exercise 5</t>
+          <t>Exercise 4</t>
         </is>
       </c>
       <c r="C68" s="4" t="inlineStr">
         <is>
-          <t>Put the test back as it was and raise the yearly cost of treating advanced cancer. How high must it be for screening from 50 to become "Dominant" (cheaper and better) in Results, section 2?</t>
+          <t>Make the test perfect (sensitivity and specificity 100%). What happens to the cost of screening (Results, section 4), and to the status of "No screening" in section 3? Why?</t>
         </is>
       </c>
     </row>
     <row r="69" ht="30" customHeight="1">
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>Exercise 6</t>
+          <t>Exercise 5</t>
         </is>
       </c>
       <c r="C69" s="4" t="inlineStr">
         <is>
-          <t>Open Trace 2 and look at age 50, when screening starts. What happens to the number of people with early cancer, and to diagnoses? Section 6 of Results shows the same in incidence.</t>
+          <t>Put the test back as it was and raise the yearly cost of treating advanced cancer. How high must it be for screening from 50 to become "Dominant" (cheaper and better) in Results, section 2?</t>
         </is>
       </c>
     </row>
     <row r="70" ht="30" customHeight="1">
       <c r="B70" s="5" t="inlineStr">
         <is>
+          <t>Exercise 6</t>
+        </is>
+      </c>
+      <c r="C70" s="4" t="inlineStr">
+        <is>
+          <t>Open Trace 2 and look at age 50, when screening starts. What happens to the number of people with early cancer, and to diagnoses? Section 6 of Results shows the same in incidence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="30" customHeight="1">
+      <c r="B71" s="5" t="inlineStr">
+        <is>
           <t>Exercise 7</t>
         </is>
       </c>
-      <c r="C70" s="4" t="inlineStr">
+      <c r="C71" s="4" t="inlineStr">
         <is>
           <t>Change strategy 3 to screen from 40 to 84. Is it still on the efficiency frontier? Is it cost-effective?</t>
         </is>
       </c>
     </row>
-    <row r="71" ht="43.5" customHeight="1">
-      <c r="B71" s="5" t="inlineStr">
+    <row r="72" ht="43.5" customHeight="1">
+      <c r="B72" s="5" t="inlineStr">
         <is>
           <t>Exercise 8</t>
         </is>
       </c>
-      <c r="C71" s="4" t="inlineStr">
+      <c r="C72" s="4" t="inlineStr">
         <is>
           <t>Make strategy 2 a short programme that screens only from 50 to 52. Why does it become "Extendedly dominated" in Results, section 3? (Hint: compare its ICER with that of strategy 3.) Then try 70 to 74 instead: why is a short programme at the end of the age range so efficient?</t>
         </is>
       </c>
     </row>
-    <row r="72" ht="30" customHeight="1">
-      <c r="B72" s="5" t="inlineStr">
+    <row r="73" ht="30" customHeight="1">
+      <c r="B73" s="5" t="inlineStr">
         <is>
           <t>Exercise 9</t>
         </is>
       </c>
-      <c r="C72" s="4" t="inlineStr">
+      <c r="C73" s="4" t="inlineStr">
         <is>
           <t>Set the probability that treatment cures an early cancer to 0%. What is left of the value of screening?</t>
         </is>
       </c>
     </row>
-    <row r="74" ht="22" customHeight="1">
-      <c r="B74" s="3" t="inlineStr">
+    <row r="75" ht="22" customHeight="1">
+      <c r="B75" s="3" t="inlineStr">
         <is>
           <t>About</t>
         </is>
       </c>
     </row>
-    <row r="75" ht="43.5" customHeight="1">
-      <c r="B75" s="4" t="inlineStr">
+    <row r="76" ht="43.5" customHeight="1">
+      <c r="B76" s="4" t="inlineStr">
         <is>
           <t>Built as an example of a cost-effectiveness model in a spreadsheet. It works in Excel and LibreOffice Calc, uses no macros, and every result is a formula you can inspect. The structure and the shortcuts taken are listed at the end of "How it works".</t>
         </is>
@@ -3603,10 +3616,1160 @@
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B75:C75"/>
+    <mergeCell ref="B76:C76"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00808080"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I45"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="58" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="12" t="inlineStr">
+        <is>
+          <t>Interface</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="13" t="inlineStr">
+        <is>
+          <t>This sheet is for programs, not for learning the model: it tells code that runs the workbook (cea_workbook.py, THALASSA) which cells are its inputs and which are its results. You can ignore it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="16" t="inlineStr">
+        <is>
+          <t>Cell: blank means the named range called Name (Formulas &gt; Name Manager). Min and Max: blank means the limits of the cell's data validation. Labels: a named range with one label per row of a table. Label and Unit of the inputs are taken from the Inputs sheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="19" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B5" s="19" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="C5" s="19" t="inlineStr">
+        <is>
+          <t>Cell</t>
+        </is>
+      </c>
+      <c r="D5" s="19" t="inlineStr">
+        <is>
+          <t>Label</t>
+        </is>
+      </c>
+      <c r="E5" s="19" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="F5" s="19" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="G5" s="19" t="inlineStr">
+        <is>
+          <t>Min</t>
+        </is>
+      </c>
+      <c r="H5" s="19" t="inlineStr">
+        <is>
+          <t>Max</t>
+        </is>
+      </c>
+      <c r="I5" s="19" t="inlineStr">
+        <is>
+          <t>Labels</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>cohort_size</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="D6" s="70" t="str">
+        <f>'Inputs'!A6</f>
+        <v>Number of people in the cohort</v>
+      </c>
+      <c r="E6" s="70" t="str">
+        <f>'Inputs'!C6</f>
+        <v>people</v>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>The cohort</t>
+        </is>
+      </c>
+      <c r="I6" s="13" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>start_age</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="D7" s="70" t="str">
+        <f>'Inputs'!A7</f>
+        <v>Age of the cohort at the start</v>
+      </c>
+      <c r="E7" s="70" t="str">
+        <f>'Inputs'!C7</f>
+        <v>years</v>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>The cohort</t>
+        </is>
+      </c>
+      <c r="I7" s="13" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t>p_detect_symptoms</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="D8" s="70" t="str">
+        <f>'Inputs'!A11</f>
+        <v>Early cancer found because of symptoms</v>
+      </c>
+      <c r="E8" s="70" t="str">
+        <f>'Inputs'!C11</f>
+        <v>per year</v>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>Natural history of the cancer (probabilities per year)</t>
+        </is>
+      </c>
+      <c r="I8" s="13" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>p_progression</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="D9" s="70" t="str">
+        <f>'Inputs'!A12</f>
+        <v>Undiagnosed early cancer becomes advanced</v>
+      </c>
+      <c r="E9" s="70" t="str">
+        <f>'Inputs'!C12</f>
+        <v>per year</v>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>Natural history of the cancer (probabilities per year)</t>
+        </is>
+      </c>
+      <c r="I9" s="13" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t>p_cure_early</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="D10" s="70" t="str">
+        <f>'Inputs'!A13</f>
+        <v>Treatment of an early cancer cures it</v>
+      </c>
+      <c r="E10" s="70" t="str">
+        <f>'Inputs'!C13</f>
+        <v>probability</v>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>Natural history of the cancer (probabilities per year)</t>
+        </is>
+      </c>
+      <c r="I10" s="13" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>p_death_advanced</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="D11" s="70" t="str">
+        <f>'Inputs'!A14</f>
+        <v>Death from advanced cancer</v>
+      </c>
+      <c r="E11" s="70" t="str">
+        <f>'Inputs'!C14</f>
+        <v>per year</v>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>Natural history of the cancer (probabilities per year)</t>
+        </is>
+      </c>
+      <c r="I11" s="13" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>screen_participation</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="D12" s="70" t="str">
+        <f>'Inputs'!A18</f>
+        <v>People who take the test when invited</v>
+      </c>
+      <c r="E12" s="70" t="str">
+        <f>'Inputs'!C18</f>
+        <v>proportion</v>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>Screening test</t>
+        </is>
+      </c>
+      <c r="I12" s="13" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>screen_sensitivity</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="D13" s="70" t="str">
+        <f>'Inputs'!A19</f>
+        <v>Sensitivity for early cancer</v>
+      </c>
+      <c r="E13" s="70" t="str">
+        <f>'Inputs'!C19</f>
+        <v>proportion</v>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>Screening test</t>
+        </is>
+      </c>
+      <c r="I13" s="13" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>screen_specificity</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="D14" s="70" t="str">
+        <f>'Inputs'!A20</f>
+        <v>Specificity</v>
+      </c>
+      <c r="E14" s="70" t="str">
+        <f>'Inputs'!C20</f>
+        <v>proportion</v>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>Screening test</t>
+        </is>
+      </c>
+      <c r="I14" s="13" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="13" t="inlineStr">
+        <is>
+          <t>cost_screen_test</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="D15" s="70" t="str">
+        <f>'Inputs'!A24</f>
+        <v>One screening test</v>
+      </c>
+      <c r="E15" s="70" t="str">
+        <f>'Inputs'!C24</f>
+        <v>€ per test</v>
+      </c>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>Costs (€)</t>
+        </is>
+      </c>
+      <c r="I15" s="13" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="13" t="inlineStr">
+        <is>
+          <t>cost_followup_test</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="D16" s="70" t="str">
+        <f>'Inputs'!A25</f>
+        <v>One follow-up diagnostic test after a positive screen</v>
+      </c>
+      <c r="E16" s="70" t="str">
+        <f>'Inputs'!C25</f>
+        <v>€ per follow-up test</v>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>Costs (€)</t>
+        </is>
+      </c>
+      <c r="I16" s="13" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="13" t="inlineStr">
+        <is>
+          <t>cost_early_treatment</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="D17" s="70" t="str">
+        <f>'Inputs'!A26</f>
+        <v>Treating an early cancer</v>
+      </c>
+      <c r="E17" s="70" t="str">
+        <f>'Inputs'!C26</f>
+        <v>€ per cancer, once</v>
+      </c>
+      <c r="F17" s="7" t="inlineStr">
+        <is>
+          <t>Costs (€)</t>
+        </is>
+      </c>
+      <c r="I17" s="13" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="13" t="inlineStr">
+        <is>
+          <t>cost_advanced_year</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="D18" s="70" t="str">
+        <f>'Inputs'!A27</f>
+        <v>Treating advanced cancer</v>
+      </c>
+      <c r="E18" s="70" t="str">
+        <f>'Inputs'!C27</f>
+        <v>€ per person per year</v>
+      </c>
+      <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t>Costs (€)</t>
+        </is>
+      </c>
+      <c r="I18" s="13" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="13" t="inlineStr">
+        <is>
+          <t>u_healthy</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="D19" s="70" t="str">
+        <f>'Inputs'!A31</f>
+        <v>A year without cancer</v>
+      </c>
+      <c r="E19" s="70" t="str">
+        <f>'Inputs'!C31</f>
+        <v>utility</v>
+      </c>
+      <c r="F19" s="7" t="inlineStr">
+        <is>
+          <t>Quality of life (utility weights: 0 = dead, 1 = full health)</t>
+        </is>
+      </c>
+      <c r="I19" s="13" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="13" t="inlineStr">
+        <is>
+          <t>u_early</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="D20" s="70" t="str">
+        <f>'Inputs'!A32</f>
+        <v>A year with undiagnosed early cancer</v>
+      </c>
+      <c r="E20" s="70" t="str">
+        <f>'Inputs'!C32</f>
+        <v>utility</v>
+      </c>
+      <c r="F20" s="7" t="inlineStr">
+        <is>
+          <t>Quality of life (utility weights: 0 = dead, 1 = full health)</t>
+        </is>
+      </c>
+      <c r="I20" s="13" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="13" t="inlineStr">
+        <is>
+          <t>u_advanced</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="D21" s="70" t="str">
+        <f>'Inputs'!A33</f>
+        <v>A year with advanced cancer</v>
+      </c>
+      <c r="E21" s="70" t="str">
+        <f>'Inputs'!C33</f>
+        <v>utility</v>
+      </c>
+      <c r="F21" s="7" t="inlineStr">
+        <is>
+          <t>Quality of life (utility weights: 0 = dead, 1 = full health)</t>
+        </is>
+      </c>
+      <c r="I21" s="13" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="13" t="inlineStr">
+        <is>
+          <t>disc_costs</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="D22" s="70" t="str">
+        <f>'Inputs'!A37</f>
+        <v>Discount rate for costs</v>
+      </c>
+      <c r="E22" s="70" t="str">
+        <f>'Inputs'!C37</f>
+        <v>per year</v>
+      </c>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t>Discounting and the decision rule</t>
+        </is>
+      </c>
+      <c r="I22" s="13" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="13" t="inlineStr">
+        <is>
+          <t>disc_effects</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="D23" s="70" t="str">
+        <f>'Inputs'!A38</f>
+        <v>Discount rate for health effects</v>
+      </c>
+      <c r="E23" s="70" t="str">
+        <f>'Inputs'!C38</f>
+        <v>per year</v>
+      </c>
+      <c r="F23" s="7" t="inlineStr">
+        <is>
+          <t>Discounting and the decision rule</t>
+        </is>
+      </c>
+      <c r="I23" s="13" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="13" t="inlineStr">
+        <is>
+          <t>wtp</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="D24" s="70" t="str">
+        <f>'Inputs'!A39</f>
+        <v>Willingness to pay per QALY gained</v>
+      </c>
+      <c r="E24" s="70" t="str">
+        <f>'Inputs'!C39</f>
+        <v>€ per QALY</v>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>Discounting and the decision rule</t>
+        </is>
+      </c>
+      <c r="I24" s="13" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="13" t="inlineStr">
+        <is>
+          <t>p_background_death</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="D25" s="70" t="str">
+        <f>'Inputs'!C42</f>
+        <v>Death from other causes</v>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>per year</t>
+        </is>
+      </c>
+      <c r="F25" s="7" t="inlineStr">
+        <is>
+          <t>Probabilities that depend on age (per year)</t>
+        </is>
+      </c>
+      <c r="I25" s="13" t="inlineStr">
+        <is>
+          <t>age_band_label</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="13" t="inlineStr">
+        <is>
+          <t>p_cancer_onset</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="D26" s="70" t="str">
+        <f>'Inputs'!D42</f>
+        <v>Cancer starts (healthy people)</v>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>per year</t>
+        </is>
+      </c>
+      <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>Probabilities that depend on age (per year)</t>
+        </is>
+      </c>
+      <c r="I26" s="13" t="inlineStr">
+        <is>
+          <t>age_band_label</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="13" t="inlineStr">
+        <is>
+          <t>strategy_name</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="D27" s="70" t="str">
+        <f>'Inputs'!A58</f>
+        <v>Strategy name</v>
+      </c>
+      <c r="E27" s="7" t="n"/>
+      <c r="F27" s="7" t="inlineStr">
+        <is>
+          <t>The strategies being compared</t>
+        </is>
+      </c>
+      <c r="I27" s="13" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="13" t="inlineStr">
+        <is>
+          <t>strategy_screens</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="D28" s="70" t="str">
+        <f>'Inputs'!C58</f>
+        <v>Screens? (Yes/No)</v>
+      </c>
+      <c r="E28" s="7" t="n"/>
+      <c r="F28" s="7" t="inlineStr">
+        <is>
+          <t>The strategies being compared</t>
+        </is>
+      </c>
+      <c r="I28" s="13" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="13" t="inlineStr">
+        <is>
+          <t>strategy_first_age</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="D29" s="70" t="str">
+        <f>'Inputs'!D58</f>
+        <v>First age screened</v>
+      </c>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>years</t>
+        </is>
+      </c>
+      <c r="F29" s="7" t="inlineStr">
+        <is>
+          <t>The strategies being compared</t>
+        </is>
+      </c>
+      <c r="I29" s="13" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="13" t="inlineStr">
+        <is>
+          <t>strategy_last_age</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="D30" s="70" t="str">
+        <f>'Inputs'!E58</f>
+        <v>Last age screened</v>
+      </c>
+      <c r="E30" s="7" t="inlineStr">
+        <is>
+          <t>years</t>
+        </is>
+      </c>
+      <c r="F30" s="7" t="inlineStr">
+        <is>
+          <t>The strategies being compared</t>
+        </is>
+      </c>
+      <c r="I30" s="13" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="13" t="inlineStr">
+        <is>
+          <t>out_check</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>output</t>
+        </is>
+      </c>
+      <c r="D31" s="7" t="inlineStr">
+        <is>
+          <t>Model checks ("All OK" when every check passes)</t>
+        </is>
+      </c>
+      <c r="E31" s="7" t="n"/>
+      <c r="F31" s="7" t="inlineStr">
+        <is>
+          <t>Results</t>
+        </is>
+      </c>
+      <c r="I31" s="13" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="13" t="inlineStr">
+        <is>
+          <t>out_best</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>output</t>
+        </is>
+      </c>
+      <c r="D32" s="7" t="inlineStr">
+        <is>
+          <t>Conclusion: the cost-effective strategy</t>
+        </is>
+      </c>
+      <c r="E32" s="7" t="n"/>
+      <c r="F32" s="7" t="inlineStr">
+        <is>
+          <t>Results</t>
+        </is>
+      </c>
+      <c r="I32" s="13" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="13" t="inlineStr">
+        <is>
+          <t>out_strategy</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>output</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t>Strategy, one row per strategy</t>
+        </is>
+      </c>
+      <c r="E33" s="7" t="n"/>
+      <c r="F33" s="7" t="inlineStr">
+        <is>
+          <t>Results</t>
+        </is>
+      </c>
+      <c r="I33" s="13" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="13" t="inlineStr">
+        <is>
+          <t>out_cost</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>output</t>
+        </is>
+      </c>
+      <c r="D34" s="7" t="inlineStr">
+        <is>
+          <t>Cost per person (discounted)</t>
+        </is>
+      </c>
+      <c r="E34" s="7" t="inlineStr">
+        <is>
+          <t>€</t>
+        </is>
+      </c>
+      <c r="F34" s="7" t="inlineStr">
+        <is>
+          <t>Results</t>
+        </is>
+      </c>
+      <c r="I34" s="13" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="13" t="inlineStr">
+        <is>
+          <t>out_qalys</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>output</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>QALYs per person (discounted)</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="inlineStr">
+        <is>
+          <t>QALYs</t>
+        </is>
+      </c>
+      <c r="F35" s="7" t="inlineStr">
+        <is>
+          <t>Results</t>
+        </is>
+      </c>
+      <c r="I35" s="13" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="13" t="inlineStr">
+        <is>
+          <t>out_life_years</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>output</t>
+        </is>
+      </c>
+      <c r="D36" s="7" t="inlineStr">
+        <is>
+          <t>Life years per person (discounted)</t>
+        </is>
+      </c>
+      <c r="E36" s="7" t="inlineStr">
+        <is>
+          <t>years</t>
+        </is>
+      </c>
+      <c r="F36" s="7" t="inlineStr">
+        <is>
+          <t>Results</t>
+        </is>
+      </c>
+      <c r="I36" s="13" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="13" t="inlineStr">
+        <is>
+          <t>out_life_years_undiscounted</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>output</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="inlineStr">
+        <is>
+          <t>Life years per person (not discounted)</t>
+        </is>
+      </c>
+      <c r="E37" s="7" t="inlineStr">
+        <is>
+          <t>years</t>
+        </is>
+      </c>
+      <c r="F37" s="7" t="inlineStr">
+        <is>
+          <t>Results</t>
+        </is>
+      </c>
+      <c r="I37" s="13" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="13" t="inlineStr">
+        <is>
+          <t>out_nmb</t>
+        </is>
+      </c>
+      <c r="B38" s="7" t="inlineStr">
+        <is>
+          <t>output</t>
+        </is>
+      </c>
+      <c r="D38" s="7" t="inlineStr">
+        <is>
+          <t>Net monetary benefit per person</t>
+        </is>
+      </c>
+      <c r="E38" s="7" t="inlineStr">
+        <is>
+          <t>€</t>
+        </is>
+      </c>
+      <c r="F38" s="7" t="inlineStr">
+        <is>
+          <t>Results</t>
+        </is>
+      </c>
+      <c r="I38" s="13" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="13" t="inlineStr">
+        <is>
+          <t>out_icer_vs_first</t>
+        </is>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>output</t>
+        </is>
+      </c>
+      <c r="D39" s="7" t="inlineStr">
+        <is>
+          <t>ICER against strategy 1</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="inlineStr">
+        <is>
+          <t>€ per QALY</t>
+        </is>
+      </c>
+      <c r="F39" s="7" t="inlineStr">
+        <is>
+          <t>Results</t>
+        </is>
+      </c>
+      <c r="I39" s="13" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="13" t="inlineStr">
+        <is>
+          <t>out_frontier_strategy</t>
+        </is>
+      </c>
+      <c r="B40" s="7" t="inlineStr">
+        <is>
+          <t>output</t>
+        </is>
+      </c>
+      <c r="D40" s="7" t="inlineStr">
+        <is>
+          <t>Strategies sorted by cost (efficiency frontier)</t>
+        </is>
+      </c>
+      <c r="E40" s="7" t="n"/>
+      <c r="F40" s="7" t="inlineStr">
+        <is>
+          <t>Results</t>
+        </is>
+      </c>
+      <c r="I40" s="13" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="13" t="inlineStr">
+        <is>
+          <t>out_frontier_status</t>
+        </is>
+      </c>
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>output</t>
+        </is>
+      </c>
+      <c r="D41" s="7" t="inlineStr">
+        <is>
+          <t>Status on the efficiency frontier</t>
+        </is>
+      </c>
+      <c r="E41" s="7" t="n"/>
+      <c r="F41" s="7" t="inlineStr">
+        <is>
+          <t>Results</t>
+        </is>
+      </c>
+      <c r="I41" s="13" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="13" t="inlineStr">
+        <is>
+          <t>out_frontier_icer</t>
+        </is>
+      </c>
+      <c r="B42" s="7" t="inlineStr">
+        <is>
+          <t>output</t>
+        </is>
+      </c>
+      <c r="D42" s="7" t="inlineStr">
+        <is>
+          <t>ICER against the previous strategy on the frontier</t>
+        </is>
+      </c>
+      <c r="E42" s="7" t="inlineStr">
+        <is>
+          <t>€ per QALY</t>
+        </is>
+      </c>
+      <c r="F42" s="7" t="inlineStr">
+        <is>
+          <t>Results</t>
+        </is>
+      </c>
+      <c r="I42" s="13" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="13" t="inlineStr">
+        <is>
+          <t>out_cancer_deaths</t>
+        </is>
+      </c>
+      <c r="B43" s="7" t="inlineStr">
+        <is>
+          <t>output</t>
+        </is>
+      </c>
+      <c r="D43" s="7" t="inlineStr">
+        <is>
+          <t>Cancer deaths over the lifetime</t>
+        </is>
+      </c>
+      <c r="E43" s="7" t="inlineStr">
+        <is>
+          <t>per 100,000 people</t>
+        </is>
+      </c>
+      <c r="F43" s="7" t="inlineStr">
+        <is>
+          <t>Results</t>
+        </is>
+      </c>
+      <c r="I43" s="13" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="13" t="inlineStr">
+        <is>
+          <t>out_diagnoses</t>
+        </is>
+      </c>
+      <c r="B44" s="7" t="inlineStr">
+        <is>
+          <t>output</t>
+        </is>
+      </c>
+      <c r="D44" s="7" t="inlineStr">
+        <is>
+          <t>Cancers diagnosed early and advanced (one row per strategy)</t>
+        </is>
+      </c>
+      <c r="E44" s="7" t="inlineStr">
+        <is>
+          <t>per 100,000 people</t>
+        </is>
+      </c>
+      <c r="F44" s="7" t="inlineStr">
+        <is>
+          <t>Results</t>
+        </is>
+      </c>
+      <c r="I44" s="13" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="13" t="inlineStr">
+        <is>
+          <t>out_incidence</t>
+        </is>
+      </c>
+      <c r="B45" s="7" t="inlineStr">
+        <is>
+          <t>output</t>
+        </is>
+      </c>
+      <c r="D45" s="7" t="inlineStr">
+        <is>
+          <t>Cancers diagnosed by age group (one row per age group, one column per strategy)</t>
+        </is>
+      </c>
+      <c r="E45" s="7" t="inlineStr">
+        <is>
+          <t>per 100,000 person-years</t>
+        </is>
+      </c>
+      <c r="F45" s="7" t="inlineStr">
+        <is>
+          <t>Results</t>
+        </is>
+      </c>
+      <c r="I45" s="13" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Update thalassa interface and model parameters
</commit_message>
<xml_diff>
--- a/cea_model.xlsx
+++ b/cea_model.xlsx
@@ -46,6 +46,7 @@
     <definedName name="strategy_screens">'Inputs'!$C$59:$C$61</definedName>
     <definedName name="strategy_first_age">'Inputs'!$D$59:$D$61</definedName>
     <definedName name="strategy_last_age">'Inputs'!$E$59:$E$61</definedName>
+    <definedName name="strategy_description">'Inputs'!$F$59:$F$61</definedName>
     <definedName name="input_check">'Inputs'!$B$3</definedName>
     <definedName name="out_check">'Results'!$B$3</definedName>
     <definedName name="out_strategy">'Results'!$B$8:$B$10</definedName>
@@ -3630,7 +3631,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I45"/>
+  <dimension ref="A1:I46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -4371,23 +4372,22 @@
     <row r="31">
       <c r="A31" s="13" t="inlineStr">
         <is>
-          <t>out_check</t>
+          <t>strategy_description</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>output</t>
-        </is>
-      </c>
-      <c r="D31" s="7" t="inlineStr">
-        <is>
-          <t>Model checks ("All OK" when every check passes)</t>
-        </is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="D31" s="70" t="str">
+        <f>'Inputs'!F58</f>
+        <v>Description</v>
       </c>
       <c r="E31" s="7" t="n"/>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>Results</t>
+          <t>The strategies being compared</t>
         </is>
       </c>
       <c r="I31" s="13" t="n"/>
@@ -4395,7 +4395,7 @@
     <row r="32">
       <c r="A32" s="13" t="inlineStr">
         <is>
-          <t>out_best</t>
+          <t>out_check</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
@@ -4405,7 +4405,7 @@
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>Conclusion: the cost-effective strategy</t>
+          <t>Model checks ("All OK" when every check passes)</t>
         </is>
       </c>
       <c r="E32" s="7" t="n"/>
@@ -4419,7 +4419,7 @@
     <row r="33">
       <c r="A33" s="13" t="inlineStr">
         <is>
-          <t>out_strategy</t>
+          <t>out_best</t>
         </is>
       </c>
       <c r="B33" s="7" t="inlineStr">
@@ -4429,7 +4429,7 @@
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>Strategy, one row per strategy</t>
+          <t>Conclusion: the cost-effective strategy</t>
         </is>
       </c>
       <c r="E33" s="7" t="n"/>
@@ -4443,7 +4443,7 @@
     <row r="34">
       <c r="A34" s="13" t="inlineStr">
         <is>
-          <t>out_cost</t>
+          <t>out_strategy</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
@@ -4453,14 +4453,10 @@
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>Cost per person (discounted)</t>
-        </is>
-      </c>
-      <c r="E34" s="7" t="inlineStr">
-        <is>
-          <t>€</t>
-        </is>
-      </c>
+          <t>Strategy, one row per strategy</t>
+        </is>
+      </c>
+      <c r="E34" s="7" t="n"/>
       <c r="F34" s="7" t="inlineStr">
         <is>
           <t>Results</t>
@@ -4471,7 +4467,7 @@
     <row r="35">
       <c r="A35" s="13" t="inlineStr">
         <is>
-          <t>out_qalys</t>
+          <t>out_cost</t>
         </is>
       </c>
       <c r="B35" s="7" t="inlineStr">
@@ -4481,12 +4477,12 @@
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>QALYs per person (discounted)</t>
+          <t>Cost per person (discounted)</t>
         </is>
       </c>
       <c r="E35" s="7" t="inlineStr">
         <is>
-          <t>QALYs</t>
+          <t>€</t>
         </is>
       </c>
       <c r="F35" s="7" t="inlineStr">
@@ -4499,7 +4495,7 @@
     <row r="36">
       <c r="A36" s="13" t="inlineStr">
         <is>
-          <t>out_life_years</t>
+          <t>out_qalys</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
@@ -4509,12 +4505,12 @@
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>Life years per person (discounted)</t>
+          <t>QALYs per person (discounted)</t>
         </is>
       </c>
       <c r="E36" s="7" t="inlineStr">
         <is>
-          <t>years</t>
+          <t>QALYs</t>
         </is>
       </c>
       <c r="F36" s="7" t="inlineStr">
@@ -4527,7 +4523,7 @@
     <row r="37">
       <c r="A37" s="13" t="inlineStr">
         <is>
-          <t>out_life_years_undiscounted</t>
+          <t>out_life_years</t>
         </is>
       </c>
       <c r="B37" s="7" t="inlineStr">
@@ -4537,7 +4533,7 @@
       </c>
       <c r="D37" s="7" t="inlineStr">
         <is>
-          <t>Life years per person (not discounted)</t>
+          <t>Life years per person (discounted)</t>
         </is>
       </c>
       <c r="E37" s="7" t="inlineStr">
@@ -4555,7 +4551,7 @@
     <row r="38">
       <c r="A38" s="13" t="inlineStr">
         <is>
-          <t>out_nmb</t>
+          <t>out_life_years_undiscounted</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
@@ -4565,12 +4561,12 @@
       </c>
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>Net monetary benefit per person</t>
+          <t>Life years per person (not discounted)</t>
         </is>
       </c>
       <c r="E38" s="7" t="inlineStr">
         <is>
-          <t>€</t>
+          <t>years</t>
         </is>
       </c>
       <c r="F38" s="7" t="inlineStr">
@@ -4583,7 +4579,7 @@
     <row r="39">
       <c r="A39" s="13" t="inlineStr">
         <is>
-          <t>out_icer_vs_first</t>
+          <t>out_nmb</t>
         </is>
       </c>
       <c r="B39" s="7" t="inlineStr">
@@ -4593,12 +4589,12 @@
       </c>
       <c r="D39" s="7" t="inlineStr">
         <is>
-          <t>ICER against strategy 1</t>
+          <t>Net monetary benefit per person</t>
         </is>
       </c>
       <c r="E39" s="7" t="inlineStr">
         <is>
-          <t>€ per QALY</t>
+          <t>€</t>
         </is>
       </c>
       <c r="F39" s="7" t="inlineStr">
@@ -4611,7 +4607,7 @@
     <row r="40">
       <c r="A40" s="13" t="inlineStr">
         <is>
-          <t>out_frontier_strategy</t>
+          <t>out_icer_vs_first</t>
         </is>
       </c>
       <c r="B40" s="7" t="inlineStr">
@@ -4621,10 +4617,14 @@
       </c>
       <c r="D40" s="7" t="inlineStr">
         <is>
-          <t>Strategies sorted by cost (efficiency frontier)</t>
-        </is>
-      </c>
-      <c r="E40" s="7" t="n"/>
+          <t>ICER against strategy 1</t>
+        </is>
+      </c>
+      <c r="E40" s="7" t="inlineStr">
+        <is>
+          <t>€ per QALY</t>
+        </is>
+      </c>
       <c r="F40" s="7" t="inlineStr">
         <is>
           <t>Results</t>
@@ -4635,7 +4635,7 @@
     <row r="41">
       <c r="A41" s="13" t="inlineStr">
         <is>
-          <t>out_frontier_status</t>
+          <t>out_frontier_strategy</t>
         </is>
       </c>
       <c r="B41" s="7" t="inlineStr">
@@ -4645,7 +4645,7 @@
       </c>
       <c r="D41" s="7" t="inlineStr">
         <is>
-          <t>Status on the efficiency frontier</t>
+          <t>Strategies sorted by cost (efficiency frontier)</t>
         </is>
       </c>
       <c r="E41" s="7" t="n"/>
@@ -4659,7 +4659,7 @@
     <row r="42">
       <c r="A42" s="13" t="inlineStr">
         <is>
-          <t>out_frontier_icer</t>
+          <t>out_frontier_status</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr">
@@ -4669,14 +4669,10 @@
       </c>
       <c r="D42" s="7" t="inlineStr">
         <is>
-          <t>ICER against the previous strategy on the frontier</t>
-        </is>
-      </c>
-      <c r="E42" s="7" t="inlineStr">
-        <is>
-          <t>€ per QALY</t>
-        </is>
-      </c>
+          <t>Status on the efficiency frontier</t>
+        </is>
+      </c>
+      <c r="E42" s="7" t="n"/>
       <c r="F42" s="7" t="inlineStr">
         <is>
           <t>Results</t>
@@ -4687,7 +4683,7 @@
     <row r="43">
       <c r="A43" s="13" t="inlineStr">
         <is>
-          <t>out_cancer_deaths</t>
+          <t>out_frontier_icer</t>
         </is>
       </c>
       <c r="B43" s="7" t="inlineStr">
@@ -4697,12 +4693,12 @@
       </c>
       <c r="D43" s="7" t="inlineStr">
         <is>
-          <t>Cancer deaths over the lifetime</t>
+          <t>ICER against the previous strategy on the frontier</t>
         </is>
       </c>
       <c r="E43" s="7" t="inlineStr">
         <is>
-          <t>per 100,000 people</t>
+          <t>€ per QALY</t>
         </is>
       </c>
       <c r="F43" s="7" t="inlineStr">
@@ -4715,7 +4711,7 @@
     <row r="44">
       <c r="A44" s="13" t="inlineStr">
         <is>
-          <t>out_diagnoses</t>
+          <t>out_cancer_deaths</t>
         </is>
       </c>
       <c r="B44" s="7" t="inlineStr">
@@ -4725,7 +4721,7 @@
       </c>
       <c r="D44" s="7" t="inlineStr">
         <is>
-          <t>Cancers diagnosed early and advanced (one row per strategy)</t>
+          <t>Cancer deaths over the lifetime</t>
         </is>
       </c>
       <c r="E44" s="7" t="inlineStr">
@@ -4743,30 +4739,58 @@
     <row r="45">
       <c r="A45" s="13" t="inlineStr">
         <is>
+          <t>out_diagnoses</t>
+        </is>
+      </c>
+      <c r="B45" s="7" t="inlineStr">
+        <is>
+          <t>output</t>
+        </is>
+      </c>
+      <c r="D45" s="7" t="inlineStr">
+        <is>
+          <t>Cancers diagnosed early and advanced (one row per strategy)</t>
+        </is>
+      </c>
+      <c r="E45" s="7" t="inlineStr">
+        <is>
+          <t>per 100,000 people</t>
+        </is>
+      </c>
+      <c r="F45" s="7" t="inlineStr">
+        <is>
+          <t>Results</t>
+        </is>
+      </c>
+      <c r="I45" s="13" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="13" t="inlineStr">
+        <is>
           <t>out_incidence</t>
         </is>
       </c>
-      <c r="B45" s="7" t="inlineStr">
+      <c r="B46" s="7" t="inlineStr">
         <is>
           <t>output</t>
         </is>
       </c>
-      <c r="D45" s="7" t="inlineStr">
+      <c r="D46" s="7" t="inlineStr">
         <is>
           <t>Cancers diagnosed by age group (one row per age group, one column per strategy)</t>
         </is>
       </c>
-      <c r="E45" s="7" t="inlineStr">
+      <c r="E46" s="7" t="inlineStr">
         <is>
           <t>per 100,000 person-years</t>
         </is>
       </c>
-      <c r="F45" s="7" t="inlineStr">
+      <c r="F46" s="7" t="inlineStr">
         <is>
           <t>Results</t>
         </is>
       </c>
-      <c r="I45" s="13" t="n"/>
+      <c r="I46" s="13" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5322,7 +5346,7 @@
         </is>
       </c>
       <c r="B3" s="15" t="str">
-        <f>IF(AND(MIN(B6)&gt;=1,MAX(B6)&lt;=10000000,MIN(B7)&gt;=40,MAX(B7)&lt;=80,MIN(B11)&gt;=0,MAX(B11)&lt;=1,MIN(B12)&gt;=0,MAX(B12)&lt;=1,MIN(B13)&gt;=0,MAX(B13)&lt;=1,MIN(B14)&gt;=0,MAX(B14)&lt;=1,MIN(B18)&gt;=0,MAX(B18)&lt;=1,MIN(B19)&gt;=0,MAX(B19)&lt;=1,MIN(B20)&gt;=0,MAX(B20)&lt;=1,MIN(B24)&gt;=0,MIN(B25)&gt;=0,MIN(B26)&gt;=0,MIN(B27)&gt;=0,MIN(B31)&gt;=0,MAX(B31)&lt;=1,MIN(B32)&gt;=0,MAX(B32)&lt;=1,MIN(B33)&gt;=0,MAX(B33)&lt;=1,MIN(B37)&gt;=0,MAX(B37)&lt;=0.2,MIN(B38)&gt;=0,MAX(B38)&lt;=0.2,MIN(B39)&gt;=0,MIN(C43:D54)&gt;=0,MAX(C43:D54)&lt;=1),"OK","CHECK")</f>
+        <f>IF(AND(MIN(B6)&gt;=1,MAX(B6)&lt;=10000000,MIN(B7)&gt;=40,MAX(B7)&lt;=80,MIN(B11)&gt;=0,MAX(B11)&lt;=1,MIN(B12)&gt;=0,MAX(B12)&lt;=1,MIN(B13)&gt;=0,MAX(B13)&lt;=1,MIN(B14)&gt;=0,MAX(B14)&lt;=1,MIN(B18)&gt;=0,MAX(B18)&lt;=1,MIN(B19)&gt;=0,MAX(B19)&lt;=1,MIN(B20)&gt;=0,MAX(B20)&lt;=1,MIN(B24)&gt;=0,MIN(B25)&gt;=0,MIN(B26)&gt;=0,MIN(B27)&gt;=0,MIN(B31)&gt;=0,MAX(B31)&lt;=1,MIN(B32)&gt;=0,MAX(B32)&lt;=1,MIN(B33)&gt;=0,MAX(B33)&lt;=1,MIN(B37)&gt;=0,MAX(B37)&lt;=1,MIN(B38)&gt;=0,MAX(B38)&lt;=1,MIN(B39)&gt;=0,MIN(C43:D54)&gt;=0,MAX(C43:D54)&lt;=1),"OK","CHECK")</f>
         <v>OK</v>
       </c>
       <c r="C3" s="16" t="inlineStr">
@@ -6560,7 +6584,7 @@
       </c>
       <c r="F61" s="4" t="inlineStr">
         <is>
-          <t>The same, but screening starts five years earlier, at 45.</t>
+          <t>Everyone aged 45 to 74 is invited to a screening test every year: the same as Screening 50-74, but starting five years earlier.</t>
         </is>
       </c>
     </row>
@@ -6633,13 +6657,13 @@
       <formula1>0</formula1>
       <formula2>1</formula2>
     </dataValidation>
-    <dataValidation sqref="B37" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Not a valid value" error="Enter a number between 0 and 0.2 (for example 0.25 for 25%)." type="decimal" operator="between">
+    <dataValidation sqref="B37" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Not a valid value" error="Enter a number between 0 and 1 (for example 0.25 for 25%)." type="decimal" operator="between">
       <formula1>0</formula1>
-      <formula2>0.2</formula2>
+      <formula2>1</formula2>
     </dataValidation>
-    <dataValidation sqref="B38" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Not a valid value" error="Enter a number between 0 and 0.2 (for example 0.25 for 25%)." type="decimal" operator="between">
+    <dataValidation sqref="B38" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Not a valid value" error="Enter a number between 0 and 1 (for example 0.25 for 25%)." type="decimal" operator="between">
       <formula1>0</formula1>
-      <formula2>0.2</formula2>
+      <formula2>1</formula2>
     </dataValidation>
     <dataValidation sqref="B39" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Not a valid value" error="Enter a number that is 0 or more." type="decimal" operator="greaterThanOrEqual">
       <formula1>0</formula1>

</xml_diff>